<commit_message>
Modello 3D Collectable, Potenziamenti, Morte su pianeta
Fatto modello 3D lampeggiante degli oggetti raccoglibili. Gestita logica di morte istantanea nel caso di collisione con un pianeta. Completato sistema di potenziamenti (mancano le logiche di cosa effettivamente fanno i potenziamenti, da inserire in Enhancement Effect), che si attivano / disattivano a seconda del completamento missioni anche con i cambi scena
</commit_message>
<xml_diff>
--- a/TextFiles/Database missioni.xlsx
+++ b/TextFiles/Database missioni.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefy\Desktop\Progetto Serious Game\ProgettoSeriousGame\TextFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F2543C-B257-4C32-BC0D-5743612BCA79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AD5427-0814-41E8-8334-E668D6EF6828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="-20850" windowWidth="20090" windowHeight="14460" xr2:uid="{A01D3E12-92BC-4039-ADA7-2749234A279B}"/>
+    <workbookView xWindow="17850" yWindow="-19280" windowWidth="17410" windowHeight="12940" xr2:uid="{A01D3E12-92BC-4039-ADA7-2749234A279B}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t>Missioni</t>
   </si>
@@ -129,6 +129,21 @@
   </si>
   <si>
     <t>Recupero Dati di bordo</t>
+  </si>
+  <si>
+    <t>Potenziamenti</t>
+  </si>
+  <si>
+    <t>Radiation Shield</t>
+  </si>
+  <si>
+    <t>Music</t>
+  </si>
+  <si>
+    <t>Speed1</t>
+  </si>
+  <si>
+    <t>Armor</t>
   </si>
 </sst>
 </file>
@@ -500,20 +515,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66CEEBA-BBC5-4F9B-9447-3E2AB89B1B48}">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="18.73046875" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="17.86328125" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" customWidth="1"/>
     <col min="14" max="14" width="20.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -524,59 +541,83 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
       <c r="G5" t="s">
         <v>1</v>
       </c>
       <c r="H5" t="s">
         <v>27</v>
       </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
       <c r="M5" t="s">
         <v>1</v>
       </c>
       <c r="N5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>2</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
       <c r="G7" t="s">
         <v>10</v>
       </c>
       <c r="H7" t="s">
         <v>20</v>
       </c>
+      <c r="I7" t="s">
+        <v>34</v>
+      </c>
       <c r="M7" t="s">
         <v>21</v>
       </c>
       <c r="N7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="O7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
       </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
       <c r="G8" t="s">
         <v>23</v>
       </c>
       <c r="H8" t="s">
         <v>24</v>
       </c>
+      <c r="I8" t="s">
+        <v>33</v>
+      </c>
       <c r="M8" t="s">
         <v>29</v>
       </c>
@@ -584,23 +625,29 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>4</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>5</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -608,7 +655,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -616,7 +663,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -624,7 +671,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Aggiornamento Livello 2 e fine livello1
Livello 1:
- Aggiunti pianeti dopo il bordo

Livello 2:
- Fatti materiali, scale, missioni e posizionamento per i pianeti (mancano gli anelli di Saturno e sono finiti)
- Riposizionato i gruppi di asteroidi, e messo gli ID per le quest nuove (finiti, se vogliamo possiamo aggiungerne altre (no)
- Fatto minimappa del secondo livello
- Per le missioni, fatti gli ID di quelle nuove, quindi in teoria sono tutte pronte e funzionanti
- Aggiunto missioni per ultimi potenziamenti della navicella (manca solo quello per la fine del gioco)
</commit_message>
<xml_diff>
--- a/TextFiles/Database missioni.xlsx
+++ b/TextFiles/Database missioni.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefy\Desktop\Progetto Serious Game\ProgettoSeriousGame\TextFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AD5427-0814-41E8-8334-E668D6EF6828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354BFF0B-1B92-4B0B-99EC-7A3BFAB5034D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17850" yWindow="-19280" windowWidth="17410" windowHeight="12940" xr2:uid="{A01D3E12-92BC-4039-ADA7-2749234A279B}"/>
+    <workbookView xWindow="14317" yWindow="2925" windowWidth="14565" windowHeight="14438" xr2:uid="{A01D3E12-92BC-4039-ADA7-2749234A279B}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>Missioni</t>
   </si>
@@ -144,6 +144,18 @@
   </si>
   <si>
     <t>Armor</t>
+  </si>
+  <si>
+    <t>M_R002</t>
+  </si>
+  <si>
+    <t>M_R003</t>
+  </si>
+  <si>
+    <t>M_C002</t>
+  </si>
+  <si>
+    <t>M_C003</t>
   </si>
 </sst>
 </file>
@@ -635,6 +647,18 @@
       <c r="C9" t="s">
         <v>32</v>
       </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+      <c r="M9" t="s">
+        <v>36</v>
+      </c>
+      <c r="N9" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
@@ -645,6 +669,18 @@
       </c>
       <c r="C10" t="s">
         <v>32</v>
+      </c>
+      <c r="G10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Aggiornamento del database missioni su Excel
</commit_message>
<xml_diff>
--- a/TextFiles/Database missioni.xlsx
+++ b/TextFiles/Database missioni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefy\Desktop\Progetto Serious Game\ProgettoSeriousGame\TextFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354BFF0B-1B92-4B0B-99EC-7A3BFAB5034D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81AFFC5-BAA3-4C1D-A470-8C8913C6400F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14317" yWindow="2925" windowWidth="14565" windowHeight="14438" xr2:uid="{A01D3E12-92BC-4039-ADA7-2749234A279B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="43">
   <si>
     <t>Missioni</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>M_C003</t>
+  </si>
+  <si>
+    <t>Speed2</t>
+  </si>
+  <si>
+    <t>Magnetic Shield</t>
+  </si>
+  <si>
+    <t>Fine Gioco</t>
   </si>
 </sst>
 </file>
@@ -659,6 +668,9 @@
       <c r="N9" t="s">
         <v>22</v>
       </c>
+      <c r="O9" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
@@ -676,6 +688,9 @@
       <c r="H10" t="s">
         <v>24</v>
       </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
       <c r="M10" t="s">
         <v>37</v>
       </c>
@@ -690,6 +705,9 @@
       <c r="B11" t="s">
         <v>16</v>
       </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
@@ -698,6 +716,9 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
@@ -706,6 +727,9 @@
       <c r="B13" t="s">
         <v>18</v>
       </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
@@ -713,6 +737,9 @@
       </c>
       <c r="B14" t="s">
         <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>